<commit_message>
feat(validation): adjudicate 14 reviewer disagreements and finalise human-eval analysis
</commit_message>
<xml_diff>
--- a/results/human_eval_v2/adjudication.xlsx
+++ b/results/human_eval_v2/adjudication.xlsx
@@ -564,8 +564,16 @@
           <t>Matches gold: 5 days for CPIO decision.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Gives 10 days for third-party response + 5 days for CPIO decision, not 5 days from receipt; wrong timeline.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -623,8 +631,16 @@
           <t>States 6 days instead of 14 days</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>States the 14-day limit, cut off before 'cannot reject/amend'; second reader's '6 days' note was a misreading.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -694,8 +710,16 @@
           <t>Matches gold: within 5 days for CPIO decision.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Same as V005: 10 + 5 days instead of 5 days from receipt; contradicts gold.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -757,8 +781,16 @@
           <t>Matches gold: inactivated virus.</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>States Covaxin is inactivated virus but cut off before Covishield (adenovirus vector); one of two components, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -842,8 +874,16 @@
           <t>Matches gold: 14 days, cannot reject/amend.</t>
         </is>
       </c>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Says 'Rajya Sabha lo Money Bill amend cheyagalavu' (can amend); contradicts gold.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -906,8 +946,16 @@
           <t>Matches gold: 12 months.</t>
         </is>
       </c>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>States 12 months, cut off before the 6-month extension; part of gold, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -965,8 +1013,16 @@
           <t>States cannot amend/reject, cut off before 14 days.</t>
         </is>
       </c>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>States Rajya Sabha cannot amend/reject, cut off before the 14-day limit; part of gold, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1041,8 +1097,16 @@
           <t>Matches gold: 12 months.</t>
         </is>
       </c>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>States 12 months, no 6-month extension; part of gold, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1114,8 +1178,16 @@
           <t>Matches gold: 12 months.</t>
         </is>
       </c>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>States 12 months, no 6-month extension; part of gold, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1178,8 +1250,16 @@
           <t>Matches gold: inactivated whole-virus.</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>States Covaxin inactivated whole-virus, cut off before Covishield; one of two components, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1254,8 +1334,16 @@
           <t>Matches gold: 12 months.</t>
         </is>
       </c>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>States 12 months, no 6-month extension; part of gold, nothing contradicted.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1324,8 +1412,16 @@
           <t>Cut off early</t>
         </is>
       </c>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>CORRECT</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>States High Court has wider writ jurisdiction under Art. 226 vs Art. 32; matches gold.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1395,8 +1491,16 @@
           <t>Matches gold: 5 days.</t>
         </is>
       </c>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Same as V005: 10 + 5 days instead of 5 days from receipt; contradicts gold.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1454,8 +1558,16 @@
           <t>Cut off early</t>
         </is>
       </c>
-      <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>CORRECT</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>States High Court has wider writ jurisdiction under Art. 226; matches gold.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>